<commit_message>
docs: double AR4 motor steps for Annin 6.1+ DIP settings
</commit_message>
<xml_diff>
--- a/Robots/AR4/Axis Calculations.xlsx
+++ b/Robots/AR4/Axis Calculations.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>Drive Output Scale</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>Lag Error In Increments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor steps/rev doubled to match Annin AR4 software 6.1+ DIP settings (J1-J4/J6 400→800, J5 800→1600). M4 600→1200 keeps the existing 1.5× equivalent vs a 400-step DIP. Encoder scaling is unchanged. CODESYS PersistentVars.PulsesPerRevolution = Effective Motor Steps per Revolution.</t>
   </si>
 </sst>
 </file>
@@ -611,8 +614,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5CF762-EE50-4516-9624-ECA299F3B35B}">
-  <dimension ref="B3:R9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5CF762-EE50-4516-9624-ECA299F3B35B}">
+  <dimension ref="B3:R11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" customWidth="1"/>
@@ -676,11 +679,11 @@
         <v>40</v>
       </c>
       <c r="E4" s="13">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="F4" s="14">
         <f>D4*E4</f>
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="H4" s="10">
         <v>160000</v>
@@ -722,11 +725,11 @@
         <v>50</v>
       </c>
       <c r="E5" s="13">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="F5" s="14">
         <f t="shared" ref="F5:F9" si="2">D5*E5</f>
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="H5" s="10">
         <v>200000</v>
@@ -768,11 +771,11 @@
         <v>50</v>
       </c>
       <c r="E6" s="13">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="F6" s="14">
         <f t="shared" si="2"/>
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="H6" s="10">
         <v>200000</v>
@@ -815,11 +818,11 @@
         <v>44.8</v>
       </c>
       <c r="E7" s="13">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="F7" s="14">
         <f t="shared" si="2"/>
-        <v>26880</v>
+        <v>53760</v>
       </c>
       <c r="H7" s="10">
         <v>4000</v>
@@ -862,11 +865,11 @@
         <v>9.8125</v>
       </c>
       <c r="E8" s="13">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="F8" s="14">
         <f t="shared" si="2"/>
-        <v>7850</v>
+        <v>15700</v>
       </c>
       <c r="H8" s="10">
         <v>38270</v>
@@ -909,11 +912,11 @@
         <v>20.203125</v>
       </c>
       <c r="E9" s="13">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="F9" s="14">
         <f t="shared" si="2"/>
-        <v>8081.25</v>
+        <v>16162.5</v>
       </c>
       <c r="H9" s="11">
         <v>4000</v>
@@ -945,6 +948,11 @@
       <c r="R9" s="12">
         <f>Q9*O9</f>
         <v>4489.5833333333339</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18">
+      <c r="B11" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -954,7 +962,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AFD2E7A-B27D-4E92-84C9-38B140952E34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AFD2E7A-B27D-4E92-84C9-38B140952E34}">
   <dimension ref="B5:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1032,15 +1040,15 @@
         <v>40</v>
       </c>
       <c r="F7" s="1">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="G7" s="4">
         <f>E7*F7</f>
-        <v>16000</v>
+        <v>32000</v>
       </c>
       <c r="H7" s="5">
         <f t="shared" ref="H7:H12" si="0">(D7/G7)*C7</f>
-        <v>737.25749999999994</v>
+        <v>368.62875</v>
       </c>
       <c r="J7" s="1">
         <v>4000</v>
@@ -1068,15 +1076,15 @@
         <v>50</v>
       </c>
       <c r="F8" s="1">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" ref="G8:G12" si="2">E8*F8</f>
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="H8" s="5">
         <f t="shared" si="0"/>
-        <v>589.80599999999993</v>
+        <v>294.903</v>
       </c>
       <c r="J8" s="1">
         <v>4000</v>
@@ -1104,15 +1112,15 @@
         <v>50</v>
       </c>
       <c r="F9" s="1">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="G9" s="4">
         <f t="shared" si="2"/>
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="H9" s="5">
         <f t="shared" si="0"/>
-        <v>589.80599999999993</v>
+        <v>294.903</v>
       </c>
       <c r="J9" s="1">
         <v>4000</v>
@@ -1141,15 +1149,15 @@
         <v>44.8</v>
       </c>
       <c r="F10" s="1">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>26880</v>
+        <v>53760</v>
       </c>
       <c r="H10" s="5">
         <f t="shared" si="0"/>
-        <v>438.84375</v>
+        <v>219.421875</v>
       </c>
       <c r="J10" s="1">
         <v>4000</v>
@@ -1178,15 +1186,15 @@
         <v>9.8125</v>
       </c>
       <c r="F11" s="1">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>7850</v>
+        <v>15700</v>
       </c>
       <c r="H11" s="5">
         <f t="shared" si="0"/>
-        <v>1502.6904458598724</v>
+        <v>751.3452229299363</v>
       </c>
       <c r="J11" s="1">
         <v>4000</v>
@@ -1215,15 +1223,15 @@
         <v>20.203125</v>
       </c>
       <c r="F12" s="1">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>8081.25</v>
+        <v>16162.5</v>
       </c>
       <c r="H12" s="5">
         <f t="shared" si="0"/>
-        <v>1459.6900232018561</v>
+        <v>729.8450116009281</v>
       </c>
       <c r="J12" s="1">
         <v>4000</v>
@@ -1235,6 +1243,11 @@
       <c r="L12" s="6">
         <f t="shared" si="3"/>
         <v>4.4547563805104407E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13">
+      <c r="B14" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: AR4 6.1 microsteps with J4 at 800 and matching PulsesPerRevolution
</commit_message>
<xml_diff>
--- a/Robots/AR4/Axis Calculations.xlsx
+++ b/Robots/AR4/Axis Calculations.xlsx
@@ -111,7 +111,7 @@
     <t>Lag Error In Increments</t>
   </si>
   <si>
-    <t xml:space="preserve">Motor steps/rev doubled to match Annin AR4 software 6.1+ DIP settings (J1-J4/J6 400→800, J5 800→1600). M4 600→1200 keeps the existing 1.5× equivalent vs a 400-step DIP. Encoder scaling is unchanged. CODESYS PersistentVars.PulsesPerRevolution = Effective Motor Steps per Revolution.</t>
+    <t xml:space="preserve">Motor steps/rev match Annin AR4 software 6.1+ DIP settings (J1-J4/J6 800, J5 1600). Encoder scaling is unchanged. CODESYS PersistentVars.PulsesPerRevolution = Effective Motor Steps per Revolution.</t>
   </si>
 </sst>
 </file>
@@ -818,11 +818,11 @@
         <v>44.8</v>
       </c>
       <c r="E7" s="13">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="F7" s="14">
         <f t="shared" si="2"/>
-        <v>53760</v>
+        <v>35840</v>
       </c>
       <c r="H7" s="10">
         <v>4000</v>
@@ -1149,15 +1149,15 @@
         <v>44.8</v>
       </c>
       <c r="F10" s="1">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>53760</v>
+        <v>35840</v>
       </c>
       <c r="H10" s="5">
         <f t="shared" si="0"/>
-        <v>219.421875</v>
+        <v>329.1328125</v>
       </c>
       <c r="J10" s="1">
         <v>4000</v>

</xml_diff>